<commit_message>
Update the project pages and reports with the corrected and extended analyses
</commit_message>
<xml_diff>
--- a/projects/trial-results-audit/downloads/trial_results_audit_tables.xlsx
+++ b/projects/trial-results-audit/downloads/trial_results_audit_tables.xlsx
@@ -30,6 +30,8 @@
     <sheet name="Post hoc flat spread" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="Post hoc analysis order" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="Worked example" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Post hoc A4 consequence" sheetId="24" state="visible" r:id="rId26"/>
+    <sheet name="Post hoc A4 cell flow" sheetId="25" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -439,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -587,6 +589,18 @@
       <c r="B12" t="inlineStr">
         <is>
           <t>ClinicalTrials.gov, U.S. National Library of Medicine. Modifications are described in the denominator rules and the data dictionary (Additional files 1 and 2 of the article; docs/rules.md and docs/data_dictionary.csv in the source archive).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Amendment 4</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Sheets 'Post hoc A4 consequence' and 'Post hoc A4 cell flow' (added 24 October 2026) report the arm-differential consequence analysis of amendment 4 (Additional file 1, Parts C and D), run once on 24 October 2026 after all other results were known. A comparison cell is one row and category of an outcome with exactly two groups; it is affected when at least one arm's row-level number analyzed differs from its outcome-level count. Source: results/tables/heldout_posthoc_A4/consequence/ in Additional file 3.</t>
         </is>
       </c>
     </row>
@@ -2695,7 +2709,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SQL and independent R tier, rule and denominators agree</t>
+          <t>SQL and R reference tier, rule and denominators agree</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -2721,7 +2735,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SQL and independent R outcome-group tier and rules agree</t>
+          <t>SQL and R reference outcome-group tier and rules agree</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -6674,6 +6688,1211 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="70" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>measure</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>numerator</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>denominator</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>risk-difference interval changes its relation to 0</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>all affected cells; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>21</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1052</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>absolute change in risk difference above 1 percentage point</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>all affected cells; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>358</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1052</v>
+      </c>
+      <c r="F3" t="n">
+        <v>34.0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>absolute change in risk difference above 5 percentage points</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>all affected cells; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>98</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1052</v>
+      </c>
+      <c r="F4" t="n">
+        <v>9.3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>risk ratio changes by 10% or more (both counts above 0)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>all affected cells; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>141</v>
+      </c>
+      <c r="E5" t="n">
+        <v>714</v>
+      </c>
+      <c r="F5" t="n">
+        <v>19.7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>risk-difference interval changes its relation to 0</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>primary outcomes; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>149</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>absolute change in risk difference above 1 percentage point</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>primary outcomes; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>58</v>
+      </c>
+      <c r="E7" t="n">
+        <v>149</v>
+      </c>
+      <c r="F7" t="n">
+        <v>38.9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>absolute change in risk difference above 5 percentage points</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>primary outcomes; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>14</v>
+      </c>
+      <c r="E8" t="n">
+        <v>149</v>
+      </c>
+      <c r="F8" t="n">
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>risk ratio changes by 10% or more (both counts above 0)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>primary outcomes; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>12</v>
+      </c>
+      <c r="E9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F9" t="n">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>risk-difference interval changes its relation to 0</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>without NCT02443155; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>21</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1034</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>absolute change in risk difference above 1 percentage point</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>without NCT02443155; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>347</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1034</v>
+      </c>
+      <c r="F11" t="n">
+        <v>33.6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>absolute change in risk difference above 5 percentage points</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>without NCT02443155; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>95</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1034</v>
+      </c>
+      <c r="F12" t="n">
+        <v>9.2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>risk ratio changes by 10% or more (both counts above 0)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>without NCT02443155; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>136</v>
+      </c>
+      <c r="E13" t="n">
+        <v>700</v>
+      </c>
+      <c r="F13" t="n">
+        <v>19.4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>risk-difference interval changes its relation to 0</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>without the ten largest contributors; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>18</v>
+      </c>
+      <c r="E14" t="n">
+        <v>849</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>absolute change in risk difference above 1 percentage point</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>without the ten largest contributors; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>287</v>
+      </c>
+      <c r="E15" t="n">
+        <v>849</v>
+      </c>
+      <c r="F15" t="n">
+        <v>33.8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>absolute change in risk difference above 5 percentage points</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>without the ten largest contributors; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>80</v>
+      </c>
+      <c r="E16" t="n">
+        <v>849</v>
+      </c>
+      <c r="F16" t="n">
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>risk ratio changes by 10% or more (both counts above 0)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>without the ten largest contributors; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>97</v>
+      </c>
+      <c r="E17" t="n">
+        <v>573</v>
+      </c>
+      <c r="F17" t="n">
+        <v>16.9</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>median absolute change in risk difference, percentage points (Q1; Q3 in the next two rows)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>all affected cells; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0.3709</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1052</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>first quartile of the absolute change in risk difference, percentage points</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>all affected cells; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1052</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>third quartile of the absolute change in risk difference, percentage points</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>comparison cell (count of participants)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>all affected cells; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1.4466</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1052</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>whole-trial bootstrap of the interval-change share, 2.5th percentile, percent (exploratory; 2,000 replicates, seed 20261024)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>percent of comparison cells (count of participants)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>all affected cells; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>whole-trial bootstrap of the interval-change share, 97.5th percentile, percent (exploratory)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>percent of comparison cells (count of participants)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>all affected cells; heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>mean difference (standard deviation given): 95% interval changes its relation to 0</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>comparison cell (mean)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>81</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2088</v>
+      </c>
+      <c r="F23" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>mean difference: inverse-variance weight under the export divided by weight under the row-level counts, median</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>comparison cell (mean)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1.1227</v>
+      </c>
+      <c r="E24" t="n">
+        <v>2087</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>mean difference: weight ratio, first quartile</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>comparison cell (mean)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1.0526</v>
+      </c>
+      <c r="E25" t="n">
+        <v>2087</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>mean difference: weight ratio, third quartile</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>comparison cell (mean)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1.3132</v>
+      </c>
+      <c r="E26" t="n">
+        <v>2087</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>mean difference: weight more than 10% higher under the export</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>comparison cell (mean)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1157</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2087</v>
+      </c>
+      <c r="F27" t="n">
+        <v>55.4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>mean (standard error given): factor by which an SD derived as SE times square root of n is too large, median</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>arm value (mean)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1.0369</v>
+      </c>
+      <c r="E28" t="n">
+        <v>392</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>row-level count divided by outcome-level count, median</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>measurement</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>0.8389</v>
+      </c>
+      <c r="E29" t="n">
+        <v>22505</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>row-level count below half the outcome-level count</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>measurement</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>3442</v>
+      </c>
+      <c r="E30" t="n">
+        <v>22505</v>
+      </c>
+      <c r="F30" t="n">
+        <v>15.3</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>row-level count above the outcome-level count</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>measurement</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>22505</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="80" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>cells</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>differing measurements</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1 one-group outcome</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>comparison cell</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1214</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1214</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2 outcome with three or more groups</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>comparison cell</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>3952</v>
+      </c>
+      <c r="E3" t="n">
+        <v>13307</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3 two-group outcome, but the cell has a value for one group only</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>comparison cell</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>518</v>
+      </c>
+      <c r="E4" t="n">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>5 outcome analyzed in another unit</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>comparison cell</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>26</v>
+      </c>
+      <c r="E5" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>7 value not a plain number</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>comparison cell</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>9 count of participants: a denominator of 0</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>comparison cell</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>8</v>
+      </c>
+      <c r="E7" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>11 count of participants: analyzed</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>comparison cell</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1052</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1981</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>12 mean type: dispersion not a plain number</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>comparison cell</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>11</v>
+      </c>
+      <c r="E9" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>13 mean type, standard deviation: analyzed</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>comparison cell</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>2088</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3835</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>14 mean type, standard error: analyzed</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>comparison cell</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>196</v>
+      </c>
+      <c r="E11" t="n">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>15 other parameter or dispersion type (not in amendment 4, sections 4.2–4.3)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>comparison cell</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>637</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1209</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>steps with no cells: 4 tier C or D measurement; 6 missing outcome-level participant count; 8 count of participants: value not an integer, or above the row-level count; 10 count of participants: value above the outcome-level count (no proportion under the export); 12 mean type: arms differ in parameter or dispersion, or a denominator of 0</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>comparison cell</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>total affected cells</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>comparison cell</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>heldout portion, confirmed cohort (post hoc, amendment 4)</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>9706</v>
+      </c>
+      <c r="E14" t="n">
+        <v>22505</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>